<commit_message>
Added leads after april
</commit_message>
<xml_diff>
--- a/templates/template.xlsx
+++ b/templates/template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tijuanap\Programs\HSE_dashboard\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52D439A7-1006-472D-8182-CC6A671CFA7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FA4F726-6E07-4712-A6DA-C38D93BA6211}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="1560" windowWidth="23880" windowHeight="15450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-26580" yWindow="1515" windowWidth="23880" windowHeight="15450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Продажи" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="Рассчет воронки" sheetId="4" state="hidden" r:id="rId4"/>
     <sheet name="Рассчет воронки (только стади)" sheetId="5" state="hidden" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -189,7 +189,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="126">
   <si>
     <t>Программа</t>
   </si>
@@ -713,6 +713,9 @@
   </si>
   <si>
     <t>Кол-во заявок (online.hse.ru) с 1.10 по неделям</t>
+  </si>
+  <si>
+    <t>Прошлогоднее Кол-во заявок (studyonline) с 1.04</t>
   </si>
 </sst>
 </file>
@@ -2533,7 +2536,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AF1"/>
+  <dimension ref="A1:AG1"/>
   <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -2548,7 +2551,7 @@
     <col min="23" max="23" width="19.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" s="77" customFormat="1" ht="72">
+    <row r="1" spans="1:33" s="77" customFormat="1" ht="72">
       <c r="A1" s="74" t="s">
         <v>102</v>
       </c>
@@ -2644,6 +2647,9 @@
       </c>
       <c r="AF1" s="85" t="s">
         <v>119</v>
+      </c>
+      <c r="AG1" s="74" t="s">
+        <v>125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Budget calculation under development. Contracts dates seems working
</commit_message>
<xml_diff>
--- a/templates/template.xlsx
+++ b/templates/template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tijuanap\Programs\HSE_dashboard\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FA4F726-6E07-4712-A6DA-C38D93BA6211}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08494773-691E-418B-9B81-F85385B0EE37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-26580" yWindow="1515" windowWidth="23880" windowHeight="15450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Продажи" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="Рассчет воронки" sheetId="4" state="hidden" r:id="rId4"/>
     <sheet name="Рассчет воронки (только стади)" sheetId="5" state="hidden" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -189,7 +189,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="127">
   <si>
     <t>Программа</t>
   </si>
@@ -716,6 +716,9 @@
   </si>
   <si>
     <t>Прошлогоднее Кол-во заявок (studyonline) с 1.04</t>
+  </si>
+  <si>
+    <t>Регистрации в ЛК Бюджет</t>
   </si>
 </sst>
 </file>
@@ -2536,7 +2539,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AG1"/>
+  <dimension ref="A1:AH1"/>
   <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -2551,7 +2554,7 @@
     <col min="23" max="23" width="19.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" s="77" customFormat="1" ht="72">
+    <row r="1" spans="1:34" s="77" customFormat="1" ht="72">
       <c r="A1" s="74" t="s">
         <v>102</v>
       </c>
@@ -2650,6 +2653,9 @@
       </c>
       <c r="AG1" s="74" t="s">
         <v>125</v>
+      </c>
+      <c r="AH1" s="85" t="s">
+        <v>126</v>
       </c>
     </row>
   </sheetData>

</xml_diff>